<commit_message>
Update marking scheme and name list files; modify DataTable sorting and filtering behavior in index.html
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -459,14 +459,14 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>VPET and Workforce</t>
+          <t>The VTC is the largest provider of VPET in Hong Kong. Briefly explain what VPET stands for and why it is important for Hong Kong’s workforce development.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[2 marks] Correctly stating "Vocational and Professional Education and Training". [4 marks] Explaining that it focuses on practical skills or specialized trades. [4 marks] Explaining the benefit to the workforce (reducing skills gap, employment readiness). General Grading: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/irrelevant answers.
+          <t>[2 marks] Correctly stating "Vocational and Professional Education and Training". [4 marks] Explaining that it focuses on practical skills or specialized trades. [4 marks] Explaining the benefit to the workforce (reducing skills gap, employment readiness). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
 --- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the q. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -481,14 +481,14 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IVE vs. THEi</t>
+          <t>Compare IVE (Hong Kong Institute of Vocational Education) and THEi (Technological and Higher Education Institute of Hong Kong). What is the main difference between the types of qualifications/programmes offered by these two institutions?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[5 marks] Correctly identifying that IVE offers Higher Diplomas/Technical training. [5 marks] Correctly identifying that THEi offers Bachelor's Degrees. General Grading: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/irrelevant answers.
+          <t>[5 marks] Correctly identifying that IVE offers Higher Diplomas/Technical training. [5 marks] Correctly identifying that THEi offers Bachelor's Degrees. General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
 --- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the q. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -503,14 +503,14 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>"Think and Do"</t>
+          <t>VTC emphasizes the " Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[3 marks] Explaining "Think" (Theory/Academic knowledge). [3 marks] Explaining "Do" (Practical skills/Hands-on). [4 marks] Explaining the synthesis: Being able to solve problems by combining both head and hands. General Grading: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/irrelevant answers.
+          <t>[3 marks] Explaining "Think" (Theory/Academic knowledge). [3 marks] Explaining "Do" (Practical skills/Hands-on). [4 marks] Explaining the synthesis: Being able to solve problems by combining both head and hands. General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
 --- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the q. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -525,14 +525,14 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Study Pathways (Foundation)</t>
+          <t>If a Secondary 6 student does not achieve the minimum entrance requirements for a Bachelor's Degree or a Higher Diploma, what is the VTC study pathway available to them to eventually reach a Higher Diploma level? (Name the specific foundation programme).</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[5 marks] Correctly naming the "Diploma of Foundation Studies" (DFS) or "Diploma of Vocational Education" (DVE). [5 marks] Explanation of the progression (Completion of DFS guarantees/allows entry to Higher Diploma). General Grading: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/irrelevant answers.
+          <t>[5 marks] Correctly naming the "Diploma of Foundation Studies" (DFS) or "Diploma of Vocational Education" (DVE). [5 marks] Explanation of the progression (Completion of DFS guarantees/allows entry to Higher Diploma). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
 --- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the q. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -547,14 +547,14 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Industry Partnership</t>
+          <t>Why does the VTC collaborate closely with industry partners (companies and trade associations)? Give two examples of how this benefits students.</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[4 marks] General explanation (Curriculum relevance/Industry needs). [3 marks] First specific benefit (e.g., Internships). [3 marks] Second specific benefit (e.g., Job prospects or Equipment). General Grading: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/irrelevant answers.
+          <t>[4 marks] General explanation (Curriculum relevance/Industry needs). [3 marks] First specific benefit (e.g., Internships). [3 marks] Second specific benefit (e.g., Job prospects or Equipment). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
 --- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the q. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D6" t="n">

</xml_diff>

<commit_message>
Refactor scoring post-processing and email score notebooks; streamline path setup and directory creation
- Updated `step5_scoring_postporcessing.ipynb` to utilize `setup_paths` and `create_directories` from `grading_utils` for better path management.
- Improved student ID mapping logic by integrating `build_student_id_mapping` utility.
- Adjusted execution counts for cells to maintain order after refactoring.
- Enhanced performance report generation with updated data and formatting.

- Refactored `step6_email_score.ipynb` to use `setup_paths` for consistent file path handling.
- Imported `markdown_to_html` from `grading_utils` to simplify markdown conversion.
- Updated execution counts and cleaned up unused code.

- Added `markdown` package to `requirements.txt` for markdown processing.

- Deleted outdated PDF answer sheets and updated the marking scheme Excel file.

- Modified HTML template to render standard answers using markdown for better formatting.
</commit_message>
<xml_diff>
--- a/sample/VTC Test Marking Scheme.xlsx
+++ b/sample/VTC Test Marking Scheme.xlsx
@@ -464,9 +464,17 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>[2 marks] Correctly stating "Vocational and Professional Education and Training". [4 marks] Explaining that it focuses on practical skills or specialized trades. [4 marks] Explaining the benefit to the workforce (reducing skills gap, employment readiness). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
---- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+          <t>- **Definition (2 marks)**: Correctly stating "**Vocational and Professional Education and Training**".
+- **Focus (4 marks)**: Explaining that it focuses on **practical skills** or **specialized trades**.
+- **Workforce Impact (4 marks)**: Explaining the benefit to the workforce (e.g., **reducing skills gap**, **employment readiness**, supporting the economy).
+**Grading Note**: Apply the 0-10 scale rubric based on the clarity of explanation and use of terminology.
+---
+**General Grading Guide:**
+### General Rubric for Partial Marks (0-10 Scale)
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -486,9 +494,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>[5 marks] Correctly identifying that IVE offers Higher Diplomas/Technical training. [5 marks] Correctly identifying that THEi offers Bachelor's Degrees. General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
---- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+          <t>- **IVE Qualification (5 marks)**: Correctly identifying that **IVE** primarily focuses on **Higher Diploma (HD)** programmes or technical training.
+- **THEi Qualification (5 marks)**: Correctly identifying that **THEi** focuses on vocationally-oriented **Bachelor’s Degree** programmes.
+**Grading Note**: Full marks require identifying both specific qualification types. Partial marks (6-8) if one is vague.
+---
+**General Grading Guide:**
+### General Rubric for Partial Marks (0-10 Scale)
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -503,14 +518,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>VTC emphasizes the " Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
+          <t>VTC emphasizes the "Think and Do" approach. Explain what this phrase means in the context of a student's learning experience.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>[3 marks] Explaining "Think" (Theory/Academic knowledge). [3 marks] Explaining "Do" (Practical skills/Hands-on). [4 marks] Explaining the synthesis: Being able to solve problems by combining both head and hands. General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
---- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+          <t>- **"Think" Component (3 marks)**: Explaining the focus on **theory** or **academic knowledge**.
+- **"Do" Component (3 marks)**: Explaining the focus on **practical skills** or **hands-on** execution.
+- **Synthesis (4 marks)**: Explaining the integration of both (e.g., **solving problems** by combining head and hands).
+**Grading Note**: A score of 9-10 requires a clear explanation of how the two components work together.
+---
+**General Grading Guide:**
+### General Rubric for Partial Marks (0-10 Scale)
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -530,9 +553,16 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>[5 marks] Correctly naming the "Diploma of Foundation Studies" (DFS) or "Diploma of Vocational Education" (DVE). [5 marks] Explanation of the progression (Completion of DFS guarantees/allows entry to Higher Diploma). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
---- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+          <t>- **Programme Identification (5 marks)**: Correctly naming the "**Diploma of Foundation Studies**" (DFS) or "**Diploma of Vocational Education**" (DVE).
+- **Progression Pathway (5 marks)**: Explaining that successful completion allows/guarantees entry to **Higher Diploma (HD)** programmes.
+**Grading Note**: If the student misses the specific name but describes the pathway, award 3-5 marks.
+---
+**General Grading Guide:**
+### General Rubric for Partial Marks (0-10 Scale)
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -552,9 +582,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>[4 marks] General explanation (Curriculum relevance/Industry needs). [3 marks] First specific benefit (e.g., Internships). [3 marks] Second specific benefit (e.g., Job prospects or Equipment). General Rubric: 9-10 marks for complete/accurate answers; 6-8 marks for mostly correct but missing details; 3-5 marks for basic understanding; 0-2 marks for incorrect/blank answers.
---- General Grading Guide ---
-9-10 marks: The answer is complete, accurate, uses correct terminology, and is well-explained. 6-8 marks: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague. 3-5 marks: The student shows basic understanding but misses the core point or only answers half the question. 0-2 marks: The answer is largely incorrect, irrelevant, or blank.</t>
+          <t>- **General Rationale (4 marks)**: Explaining that collaboration ensures **curriculum relevance** or meets **market trends/industry needs**.
+- **Benefit Example 1 (3 marks)**: e.g., **Internships** or Work-integrated learning.
+- **Benefit Example 2 (3 marks)**: e.g., **Job placement support** or access to **industry-standard equipment**.
+**Grading Note**: To achieve 9-10 marks, the student must provide two distinct and valid benefits.
+---
+**General Grading Guide:**
+### General Rubric for Partial Marks (0-10 Scale)
+- **9-10 marks**: The answer is complete, accurate, uses correct terminology, and is well-explained.
+- **6-8 marks**: The answer is mostly correct but misses a specific detail (e.g., forgets the full name of a diploma) or the explanation is slightly vague.
+- **3-5 marks**: The student shows basic understanding but misses the core point or only answers half the question.
+- **0-2 marks**: The answer is largely incorrect, irrelevant, or blank.</t>
         </is>
       </c>
       <c r="D6" t="n">

</xml_diff>